<commit_message>
temporary commit, added multiIO rendering support for transient response
</commit_message>
<xml_diff>
--- a/apps_MAK_PPO/RPA_3species_5rxns/RPA_3species_5rxns_MAK_PPO.xlsx
+++ b/apps_MAK_PPO/RPA_3species_5rxns/RPA_3species_5rxns_MAK_PPO.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU28"/>
+  <dimension ref="A1:AX28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -652,6 +652,21 @@
           <t>2025-11-19 11:44:34</t>
         </is>
       </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>2025-11-19 12:08:19</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>2025-11-19 12:16:37</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>2025-11-19 13:00:00</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -889,6 +904,21 @@
           <t>https://www.comet.com/redsnic/rpa-3species-5rxns-mak-ppo/46bf1dbeff904d85a77106dcdddcfc7b</t>
         </is>
       </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/rpa-3species-5rxns-mak-ppo/736487f51917497a8b8d9cbbb416124f</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/rpa-3species-5rxns-mak-ppo/127823124f8e4128ac9e67ad49e00ff7</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/rpa-3species-5rxns-mak-ppo/74a97873e04f4dd9887be1e132c92f04</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1034,6 +1064,15 @@
       <c r="AU3" t="n">
         <v>5</v>
       </c>
+      <c r="AV3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AW3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AX3" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1179,6 +1218,15 @@
       <c r="AU4" t="n">
         <v>3</v>
       </c>
+      <c r="AV4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AX4" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1324,6 +1372,15 @@
       <c r="AU5" t="n">
         <v>2</v>
       </c>
+      <c r="AV5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AX5" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1469,6 +1526,15 @@
       <c r="AU6" t="n">
         <v>1280</v>
       </c>
+      <c r="AV6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="AX6" t="n">
+        <v>1280</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1614,6 +1680,15 @@
       <c r="AU7" t="b">
         <v>0</v>
       </c>
+      <c r="AV7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AW7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AX7" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1759,6 +1834,15 @@
       <c r="AU8" t="n">
         <v>0.0001</v>
       </c>
+      <c r="AV8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1904,6 +1988,15 @@
       <c r="AU9" t="n">
         <v>300</v>
       </c>
+      <c r="AV9" t="n">
+        <v>300</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>300</v>
+      </c>
+      <c r="AX9" t="n">
+        <v>300</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2049,6 +2142,15 @@
       <c r="AU10" t="n">
         <v>5</v>
       </c>
+      <c r="AV10" t="n">
+        <v>5</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>5</v>
+      </c>
+      <c r="AX10" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2194,6 +2296,15 @@
       <c r="AU11" t="n">
         <v>1024</v>
       </c>
+      <c r="AV11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="AW11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="AX11" t="n">
+        <v>1024</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2339,6 +2450,15 @@
       <c r="AU12" t="n">
         <v>10240</v>
       </c>
+      <c r="AV12" t="n">
+        <v>10240</v>
+      </c>
+      <c r="AW12" t="n">
+        <v>10240</v>
+      </c>
+      <c r="AX12" t="n">
+        <v>10240</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2484,6 +2604,15 @@
       <c r="AU13" t="n">
         <v>128</v>
       </c>
+      <c r="AV13" t="n">
+        <v>128</v>
+      </c>
+      <c r="AW13" t="n">
+        <v>128</v>
+      </c>
+      <c r="AX13" t="n">
+        <v>128</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2721,6 +2850,21 @@
           <t>{'entropy_weight': 0.001, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.001}</t>
         </is>
       </c>
+      <c r="AV14" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.02, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.02}</t>
+        </is>
+      </c>
+      <c r="AW14" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.005}</t>
+        </is>
+      </c>
+      <c r="AX14" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.01, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.01}</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2958,6 +3102,21 @@
           <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
         </is>
       </c>
+      <c r="AV15" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="AW15" t="inlineStr">
+        <is>
+          <t>{'risk': 0.97, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="AX15" t="inlineStr">
+        <is>
+          <t>{'risk': 0.97, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3103,6 +3262,15 @@
       <c r="AU16" t="n">
         <v>10</v>
       </c>
+      <c r="AV16" t="n">
+        <v>10</v>
+      </c>
+      <c r="AW16" t="n">
+        <v>10</v>
+      </c>
+      <c r="AX16" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3248,6 +3416,15 @@
       <c r="AU17" t="n">
         <v>20</v>
       </c>
+      <c r="AV17" t="n">
+        <v>20</v>
+      </c>
+      <c r="AW17" t="n">
+        <v>20</v>
+      </c>
+      <c r="AX17" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3393,6 +3570,15 @@
       <c r="AU18" t="n">
         <v>200</v>
       </c>
+      <c r="AV18" t="n">
+        <v>200</v>
+      </c>
+      <c r="AW18" t="n">
+        <v>200</v>
+      </c>
+      <c r="AX18" t="n">
+        <v>200</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3538,6 +3724,15 @@
       <c r="AU19" t="n">
         <v>1000</v>
       </c>
+      <c r="AV19" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AW19" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AX19" t="n">
+        <v>1000</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3683,6 +3878,15 @@
       <c r="AU20" t="n">
         <v>1</v>
       </c>
+      <c r="AV20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX20" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3828,6 +4032,15 @@
       <c r="AU21" t="n">
         <v>9</v>
       </c>
+      <c r="AV21" t="n">
+        <v>9</v>
+      </c>
+      <c r="AW21" t="n">
+        <v>9</v>
+      </c>
+      <c r="AX21" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4065,6 +4278,21 @@
           <t>{'type': 'lognormal_1D'}</t>
         </is>
       </c>
+      <c r="AV22" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="AW22" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="AX22" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4298,6 +4526,21 @@
         </is>
       </c>
       <c r="AU23" t="inlineStr">
+        <is>
+          <t>{'eps': 0.2, 'value_loss_weight': 0.5, 'gamma': 1, 'lam': 0.97, 'update_policy_every': 4}</t>
+        </is>
+      </c>
+      <c r="AV23" t="inlineStr">
+        <is>
+          <t>{'eps': 0.2, 'value_loss_weight': 0.5, 'gamma': 1, 'lam': 0.97, 'update_policy_every': 4}</t>
+        </is>
+      </c>
+      <c r="AW23" t="inlineStr">
+        <is>
+          <t>{'eps': 0.2, 'value_loss_weight': 0.5, 'gamma': 1, 'lam': 0.97, 'update_policy_every': 4}</t>
+        </is>
+      </c>
+      <c r="AX23" t="inlineStr">
         <is>
           <t>{'eps': 0.2, 'value_loss_weight': 0.5, 'gamma': 1, 'lam': 0.97, 'update_policy_every': 4}</t>
         </is>

</xml_diff>

<commit_message>
Restructured the excel sheet. Improved the comet presentation. Added a folder for the final results.
</commit_message>
<xml_diff>
--- a/apps_MAK_PPO/RPA_3species_5rxns/RPA_3species_5rxns_MAK_PPO.xlsx
+++ b/apps_MAK_PPO/RPA_3species_5rxns/RPA_3species_5rxns_MAK_PPO.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU28"/>
+  <dimension ref="A1:AV28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -652,6 +652,11 @@
           <t>2025-11-19 11:44:34</t>
         </is>
       </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>2025-11-19 17:34:56</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -889,6 +894,11 @@
           <t>https://www.comet.com/redsnic/rpa-3species-5rxns-mak-ppo/46bf1dbeff904d85a77106dcdddcfc7b</t>
         </is>
       </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/rpa-3species-5rxns-mak-ppo/910fe18b3e2b4b478d50f8a0de9f634e</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1034,6 +1044,9 @@
       <c r="AU3" t="n">
         <v>5</v>
       </c>
+      <c r="AV3" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1179,6 +1192,9 @@
       <c r="AU4" t="n">
         <v>3</v>
       </c>
+      <c r="AV4" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1324,6 +1340,9 @@
       <c r="AU5" t="n">
         <v>2</v>
       </c>
+      <c r="AV5" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1469,6 +1488,9 @@
       <c r="AU6" t="n">
         <v>1280</v>
       </c>
+      <c r="AV6" t="n">
+        <v>1280</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1614,6 +1636,9 @@
       <c r="AU7" t="b">
         <v>0</v>
       </c>
+      <c r="AV7" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1759,6 +1784,9 @@
       <c r="AU8" t="n">
         <v>0.0001</v>
       </c>
+      <c r="AV8" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1904,6 +1932,9 @@
       <c r="AU9" t="n">
         <v>300</v>
       </c>
+      <c r="AV9" t="n">
+        <v>300</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2049,6 +2080,9 @@
       <c r="AU10" t="n">
         <v>5</v>
       </c>
+      <c r="AV10" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2194,6 +2228,9 @@
       <c r="AU11" t="n">
         <v>1024</v>
       </c>
+      <c r="AV11" t="n">
+        <v>1024</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2339,6 +2376,9 @@
       <c r="AU12" t="n">
         <v>10240</v>
       </c>
+      <c r="AV12" t="n">
+        <v>10240</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2484,6 +2524,9 @@
       <c r="AU13" t="n">
         <v>128</v>
       </c>
+      <c r="AV13" t="n">
+        <v>128</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2721,6 +2764,11 @@
           <t>{'entropy_weight': 0.001, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.001}</t>
         </is>
       </c>
+      <c r="AV14" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.001, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.001}</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2958,6 +3006,11 @@
           <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
         </is>
       </c>
+      <c r="AV15" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3103,6 +3156,9 @@
       <c r="AU16" t="n">
         <v>10</v>
       </c>
+      <c r="AV16" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3248,6 +3304,9 @@
       <c r="AU17" t="n">
         <v>20</v>
       </c>
+      <c r="AV17" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3393,6 +3452,9 @@
       <c r="AU18" t="n">
         <v>200</v>
       </c>
+      <c r="AV18" t="n">
+        <v>200</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3538,6 +3600,9 @@
       <c r="AU19" t="n">
         <v>1000</v>
       </c>
+      <c r="AV19" t="n">
+        <v>1000</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3683,6 +3748,9 @@
       <c r="AU20" t="n">
         <v>1</v>
       </c>
+      <c r="AV20" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3828,6 +3896,9 @@
       <c r="AU21" t="n">
         <v>9</v>
       </c>
+      <c r="AV21" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4065,6 +4136,11 @@
           <t>{'type': 'lognormal_1D'}</t>
         </is>
       </c>
+      <c r="AV22" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4298,6 +4374,11 @@
         </is>
       </c>
       <c r="AU23" t="inlineStr">
+        <is>
+          <t>{'eps': 0.2, 'value_loss_weight': 0.5, 'gamma': 1, 'lam': 0.97, 'update_policy_every': 4}</t>
+        </is>
+      </c>
+      <c r="AV23" t="inlineStr">
         <is>
           <t>{'eps': 0.2, 'value_loss_weight': 0.5, 'gamma': 1, 'lam': 0.97, 'update_policy_every': 4}</t>
         </is>

</xml_diff>

<commit_message>
added soft and hard order constraint masks, fixed weights for topk entropy
</commit_message>
<xml_diff>
--- a/apps_MAK_PPO/RPA_3species_5rxns/RPA_3species_5rxns_MAK_PPO.xlsx
+++ b/apps_MAK_PPO/RPA_3species_5rxns/RPA_3species_5rxns_MAK_PPO.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX28"/>
+  <dimension ref="A1:AY28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -667,6 +667,11 @@
           <t>2025-11-19 13:00:00</t>
         </is>
       </c>
+      <c r="AY1" t="inlineStr">
+        <is>
+          <t>2025-11-21 17:17:29</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -919,6 +924,11 @@
           <t>https://www.comet.com/redsnic/rpa-3species-5rxns-mak-ppo/74a97873e04f4dd9887be1e132c92f04</t>
         </is>
       </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/rpa-3species-5rxns-mak-ppo/667c984f88a445cb80606ed75c65210c</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1073,6 +1083,9 @@
       <c r="AX3" t="n">
         <v>5</v>
       </c>
+      <c r="AY3" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1227,6 +1240,9 @@
       <c r="AX4" t="n">
         <v>3</v>
       </c>
+      <c r="AY4" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1381,6 +1397,9 @@
       <c r="AX5" t="n">
         <v>2</v>
       </c>
+      <c r="AY5" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1535,6 +1554,9 @@
       <c r="AX6" t="n">
         <v>1280</v>
       </c>
+      <c r="AY6" t="n">
+        <v>1280</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1689,6 +1711,9 @@
       <c r="AX7" t="b">
         <v>0</v>
       </c>
+      <c r="AY7" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1843,6 +1868,9 @@
       <c r="AX8" t="n">
         <v>0.0001</v>
       </c>
+      <c r="AY8" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1997,6 +2025,9 @@
       <c r="AX9" t="n">
         <v>300</v>
       </c>
+      <c r="AY9" t="n">
+        <v>300</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2151,6 +2182,9 @@
       <c r="AX10" t="n">
         <v>5</v>
       </c>
+      <c r="AY10" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2305,6 +2339,9 @@
       <c r="AX11" t="n">
         <v>1024</v>
       </c>
+      <c r="AY11" t="n">
+        <v>1024</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2459,6 +2496,9 @@
       <c r="AX12" t="n">
         <v>10240</v>
       </c>
+      <c r="AY12" t="n">
+        <v>10240</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2613,6 +2653,9 @@
       <c r="AX13" t="n">
         <v>128</v>
       </c>
+      <c r="AY13" t="n">
+        <v>128</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2865,6 +2908,11 @@
           <t>{'entropy_weight': 0.01, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.01}</t>
         </is>
       </c>
+      <c r="AY14" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.01, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.01}</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3117,6 +3165,11 @@
           <t>{'risk': 0.97, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
         </is>
       </c>
+      <c r="AY15" t="inlineStr">
+        <is>
+          <t>{'risk': 0.97, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3271,6 +3324,9 @@
       <c r="AX16" t="n">
         <v>10</v>
       </c>
+      <c r="AY16" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3425,6 +3481,9 @@
       <c r="AX17" t="n">
         <v>20</v>
       </c>
+      <c r="AY17" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3579,6 +3638,9 @@
       <c r="AX18" t="n">
         <v>200</v>
       </c>
+      <c r="AY18" t="n">
+        <v>200</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3733,6 +3795,9 @@
       <c r="AX19" t="n">
         <v>1000</v>
       </c>
+      <c r="AY19" t="n">
+        <v>1000</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3887,6 +3952,9 @@
       <c r="AX20" t="n">
         <v>1</v>
       </c>
+      <c r="AY20" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4041,6 +4109,9 @@
       <c r="AX21" t="n">
         <v>9</v>
       </c>
+      <c r="AY21" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4293,6 +4364,11 @@
           <t>{'type': 'lognormal_1D'}</t>
         </is>
       </c>
+      <c r="AY22" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4541,6 +4617,11 @@
         </is>
       </c>
       <c r="AX23" t="inlineStr">
+        <is>
+          <t>{'eps': 0.2, 'value_loss_weight': 0.5, 'gamma': 1, 'lam': 0.97, 'update_policy_every': 4}</t>
+        </is>
+      </c>
+      <c r="AY23" t="inlineStr">
         <is>
           <t>{'eps': 0.2, 'value_loss_weight': 0.5, 'gamma': 1, 'lam': 0.97, 'update_policy_every': 4}</t>
         </is>

</xml_diff>